<commit_message>
Merged MCX opTions trading OCT 23
</commit_message>
<xml_diff>
--- a/nifty_orb_agent/ORB_Agent_Reference.xlsx
+++ b/nifty_orb_agent/ORB_Agent_Reference.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="185">
   <si>
     <t xml:space="preserve">ORB Agent - Decision Source Reference</t>
   </si>
@@ -114,7 +114,7 @@
     <t xml:space="preserve">Same mirrored VWAP/volume exit as NIFTY options, independent trade book</t>
   </si>
   <si>
-    <t xml:space="preserve">MCX commodities (commodity_engine.py)</t>
+    <t xml:space="preserve">MCX commodity futures (commodity_engine.py)</t>
   </si>
   <si>
     <t xml:space="preserve">Each contract in MCX_COMMODITY_UNIVERSE - its own MCX-session opening-range candle (MCX_MARKET_OPEN_TIME, not NSE's 09:15)</t>
@@ -126,7 +126,7 @@
     <t xml:space="preserve">bootstrap.decide_todays_commodity_direction() - a SEPARATE, commodity-specific global sentiment read (gold/silver/crude/copper/natural-gas/dollar-index cues) - deliberately not the equity-cue sentiment equities/NIFTY/BANKNIFTY options use</t>
   </si>
   <si>
-    <t xml:space="preserve">N/A - the futures contract itself is bought/sold directly (MCX options are NOT used - see commodity_engine.py's docstring for why)</t>
+    <t xml:space="preserve">N/A - the futures contract itself is bought/sold directly, no strike/expiry resolution step (see MCX commodity OPTIONS row below for the options counterpart)</t>
   </si>
   <si>
     <t xml:space="preserve">The commodity future itself (every contract in the universe, no shortlist/scan filter - see 'no gain/loss-band' in the module docstring)</t>
@@ -135,7 +135,28 @@
     <t xml:space="preserve">Same mirrored VWAP/volume-MA weakness detector as equities (ADD then stop-loss)</t>
   </si>
   <si>
-    <t xml:space="preserve">Notes: "direction source" above only matters when USE_CANDLE_BASED_DIRECTION=True (candle-based mode); in sentiment mode it ignores the index entirely. The wick/quality filter (config.MAX_OR_CANDLE_WICK_PCT) is ONE shared threshold across equities, both options engines, and MCX - see config.py's comment block.</t>
+    <t xml:space="preserve">MCX commodity options (mcx_options_engine.py)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Each contract's OWN futures symbol - watched for a breakout in EITHER direction independently per commodity (NOT a shared daily bias like the futures row above)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Each contract's own futures symbol (same reasoning as NIFTY/BANKNIFTY options - MCX has no separate spot index either, so the future doubles as the strike-resolution spot reference too - index_symbol=futures_symbol)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">decide_todays_commodity_direction() - the SAME read the futures engine uses, but only gates each contract's own opening-range quality/wick filter now; does NOT pick CE vs PE for any commodity (identical demotion to NIFTY/BANKNIFTY options - see that row)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">That commodity's own futures LTP, read FRESH at signal time - shares config.OPTION_STRIKE_MODE with NIFTY/BANKNIFTY options, own MCX_OTM_STRIKES_AWAY; resolved from a SEPARATE MCX options symbol master (MCX_FO_SYMBOL_MASTER_CSV, not NSE's), filtered on each commodity's own option_underlying code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">That SAME commodity's own option (CE on an upside futures breakout, PE on a downside one) - BUY-ONLY, one NiftyOptionsEngine instance per commodity, sharing ONE trade book</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Same mirrored VWAP/volume exit as NIFTY/BANKNIFTY options, per commodity independently</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notes: "direction source" above only matters when USE_CANDLE_BASED_DIRECTION=True (candle-based mode); in sentiment mode it ignores the index entirely. The wick/quality filter (config.MAX_OR_CANDLE_WICK_PCT) is ONE shared threshold across equities, all three options engines (NIFTY/BANKNIFTY/MCX), and MCX futures - see config.py's comment block. MCX commodity futures and MCX commodity options are two completely independent engines/capital buckets/ENABLE_* flags (ENABLE_MCX_COMMODITY_TRADING / ENABLE_MCX_OPTIONS_TRADING) - either, both, or neither can be on at once.</t>
   </si>
   <si>
     <t xml:space="preserve">config.py - Key Settings by Strategy</t>
@@ -390,7 +411,7 @@
     <t xml:space="preserve">Independent capital bucket</t>
   </si>
   <si>
-    <t xml:space="preserve">MCX commodities (ENABLE_MCX_COMMODITY_TRADING = False)</t>
+    <t xml:space="preserve">MCX commodity futures (ENABLE_MCX_COMMODITY_TRADING = False)</t>
   </si>
   <si>
     <t xml:space="preserve">MCX_MARKET_OPEN_TIME</t>
@@ -417,7 +438,10 @@
     <t xml:space="preserve">MCX_CANDLE_INTERVAL_MINUTES</t>
   </si>
   <si>
-    <t xml:space="preserve">MCX's own candle size - independently configurable from NSE's</t>
+    <t xml:space="preserve">MCX's own candle size - independently configurable from NSE's; shared with MCX options below (same session)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">commodity_engine.py, mcx_options_engine.py</t>
   </si>
   <si>
     <t xml:space="preserve">MCX_COMMODITY_UNIVERSE</t>
@@ -426,13 +450,76 @@
     <t xml:space="preserve">(hand-maintained list)</t>
   </si>
   <si>
-    <t xml:space="preserve">The explicit, short list of contracts actually traded - no scan, every contract considered daily</t>
+    <t xml:space="preserve">The explicit, short list of contracts actually traded - no scan, every contract considered daily; each entry's own option_underlying is used by MCX options below</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MCX_DIRECTION_REFERENCE_SYMBOL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">None (first universe entry)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Which ONE contract's candles decide the SHARED daily direction for the whole FUTURES universe - NOT used by MCX options (see below), which decides direction per-commodity instead</t>
   </si>
   <si>
     <t xml:space="preserve">MCX_CAPITAL</t>
   </si>
   <si>
     <t xml:space="preserve">Independent capital bucket, split equally across the universe's tracked contracts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MCX commodity options (ENABLE_MCX_OPTIONS_TRADING = False)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ENABLE_MCX_OPTIONS_TRADING</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Master switch - completely independent of ENABLE_MCX_COMMODITY_TRADING (futures); enable either, both, or neither</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mcx_options_engine.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MCX_FO_SYMBOL_MASTER_CSV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data/mcx_fo_symbol_master.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MCX's OWN options instrument master - a SEPARATE file/exchange segment from NSE's NIFTY_FO_SYMBOL_MASTER_CSV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MCX_FO_MASTER_COLUMNS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(column-name mapping)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Same shape as NIFTY_FO_MASTER_COLUMNS - VERIFY against your own downloaded MCX file's real header</t>
+  </si>
+  <si>
+    <t xml:space="preserve">option_underlying (per MCX_COMMODITY_UNIVERSE entry)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">e.g. "GOLDM"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Which underlying_symbol code in MCX_FO_SYMBOL_MASTER_CSV is THIS commodity's own options - VERIFY each one; a wrong/missing value just skips that one commodity (logged), not a crash</t>
+  </si>
+  <si>
+    <t xml:space="preserve">config.py, mcx_options_engine.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MCX_OTM_STRIKES_AWAY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ONE shared strikes-away count across the whole universe - shares config.OPTION_STRIKE_MODE with NIFTY/BANKNIFTY options</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MCX_OPTIONS_CAPITAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Independent capital bucket (NOT MCX_CAPITAL, the futures bucket) - split equally across tracked commodities</t>
   </si>
   <si>
     <t xml:space="preserve">options_engine.py - Latest Changes</t>
@@ -920,7 +1007,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
@@ -1068,22 +1155,45 @@
         <v>36</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="s">
+    <row r="9" customFormat="false" ht="109.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
+      <c r="B9" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A10:G10"/>
+    <mergeCell ref="A11:G11"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1100,7 +1210,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D47"/>
+  <dimension ref="A1:D57"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
@@ -1111,7 +1221,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1119,7 +1229,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1127,7 +1237,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="B4" s="6"/>
       <c r="C4" s="6"/>
@@ -1135,161 +1245,161 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="C8" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="D8" s="4" t="s">
         <v>55</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="B17" s="6"/>
       <c r="C17" s="6"/>
@@ -1297,91 +1407,91 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="B25" s="6"/>
       <c r="C25" s="6"/>
@@ -1389,105 +1499,105 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="D30" s="4" t="s">
         <v>106</v>
-      </c>
-      <c r="B30" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="C30" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="D30" s="4" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="6" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="B34" s="6"/>
       <c r="C34" s="6"/>
@@ -1495,30 +1605,30 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1526,46 +1636,46 @@
         <v>25</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="7" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="6" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="B41" s="6"/>
       <c r="C41" s="6"/>
@@ -1573,90 +1683,210 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="7" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="7" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="B45" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="D45" s="4" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="D46" s="4" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="D47" s="4" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="D48" s="4" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="B50" s="6"/>
+      <c r="C50" s="6"/>
+      <c r="D50" s="6"/>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B51" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C51" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="C45" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="D45" s="4" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="7" t="s">
-        <v>132</v>
-      </c>
-      <c r="B46" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="C46" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="D46" s="4" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="7" t="s">
-        <v>135</v>
-      </c>
-      <c r="B47" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="C47" s="4" t="s">
-        <v>136</v>
-      </c>
-      <c r="D47" s="4" t="s">
-        <v>126</v>
+      <c r="D51" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="D52" s="4" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="D54" s="4" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="D55" s="4" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="D56" s="4" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="D57" s="4" t="s">
+        <v>151</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="8">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A4:D4"/>
@@ -1664,6 +1894,7 @@
     <mergeCell ref="A25:D25"/>
     <mergeCell ref="A34:D34"/>
     <mergeCell ref="A41:D41"/>
+    <mergeCell ref="A50:D50"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1690,75 +1921,75 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>137</v>
+        <v>166</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>138</v>
+        <v>167</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>139</v>
+        <v>168</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>140</v>
+        <v>169</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>141</v>
+        <v>170</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>142</v>
+        <v>171</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>143</v>
+        <v>172</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>144</v>
+        <v>173</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>145</v>
+        <v>174</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>146</v>
+        <v>175</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>147</v>
+        <v>176</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>148</v>
+        <v>177</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>149</v>
+        <v>178</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>150</v>
+        <v>179</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>151</v>
+        <v>180</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>152</v>
+        <v>181</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>153</v>
+        <v>182</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>154</v>
+        <v>183</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>155</v>
+        <v>184</v>
       </c>
     </row>
   </sheetData>

</xml_diff>